<commit_message>
Cambios en codigo y mpas graficas.
</commit_message>
<xml_diff>
--- a/03_outputs/03.1_descriptivas.xlsx
+++ b/03_outputs/03.1_descriptivas.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniandes-my.sharepoint.com/personal/mh_torres_uniandes_edu_co/Documents/Pregrado/8vo Semestre/01_Big_Data/03_Talleres/taller_1_grupo_05/03_outputs/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="147" documentId="11_2464E66F0BF9EA6E68D4C4C168672749E60C47D7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18C0EF66-2458-49FD-83D9-7EE62DF50556}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Train - Numéricas" sheetId="1" r:id="rId1"/>
@@ -14,7 +20,20 @@
     <sheet name="Total - Numéricas" sheetId="5" r:id="rId5"/>
     <sheet name="Total - Categóricas" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -123,8 +142,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,13 +191,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -216,7 +243,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -250,6 +277,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -284,9 +312,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -459,11 +488,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -492,7 +521,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -500,10 +529,10 @@
         <v>10263</v>
       </c>
       <c r="C2">
-        <v>38.7960635291825</v>
+        <v>38.796063529182497</v>
       </c>
       <c r="D2">
-        <v>13.27815902197739</v>
+        <v>13.278159021977389</v>
       </c>
       <c r="E2">
         <v>37</v>
@@ -521,7 +550,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -529,7 +558,7 @@
         <v>10263</v>
       </c>
       <c r="C3">
-        <v>10.49595634804638</v>
+        <v>10.495956348046381</v>
       </c>
       <c r="D3">
         <v>3.279463424644431</v>
@@ -550,7 +579,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -558,7 +587,7 @@
         <v>10263</v>
       </c>
       <c r="C4">
-        <v>47.48202280035078</v>
+        <v>47.482022800350776</v>
       </c>
       <c r="D4">
         <v>15.12197671634412</v>
@@ -579,7 +608,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -587,10 +616,10 @@
         <v>10263</v>
       </c>
       <c r="C5">
-        <v>0.4727662476858618</v>
+        <v>0.47276624768586178</v>
       </c>
       <c r="D5">
-        <v>0.4992820967986027</v>
+        <v>0.49928209679860269</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -608,7 +637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -616,7 +645,7 @@
         <v>10263</v>
       </c>
       <c r="C6">
-        <v>0.395985579265322</v>
+        <v>0.39598557926532202</v>
       </c>
       <c r="D6">
         <v>0.4890851743042301</v>
@@ -637,7 +666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -645,10 +674,10 @@
         <v>10263</v>
       </c>
       <c r="C7">
-        <v>0.2927993764006626</v>
+        <v>0.29279937640066261</v>
       </c>
       <c r="D7">
-        <v>0.4550693130759011</v>
+        <v>0.45506931307590109</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -666,7 +695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -674,10 +703,10 @@
         <v>10263</v>
       </c>
       <c r="C8">
-        <v>1592515.746932625</v>
+        <v>1592515.7469326251</v>
       </c>
       <c r="D8">
-        <v>2332537.380976002</v>
+        <v>2332537.3809760022</v>
       </c>
       <c r="E8">
         <v>990929.4375</v>
@@ -701,11 +730,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -725,9 +754,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.3303127740426776</v>
+        <v>0.33031277404267761</v>
       </c>
       <c r="B2" t="s">
         <v>20</v>
@@ -745,9 +774,9 @@
         <v>930929.4375</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.006041118581311507</v>
+        <v>6.0411185813115066E-3</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
@@ -759,15 +788,15 @@
         <v>62</v>
       </c>
       <c r="E3">
-        <v>535678.9430443548</v>
+        <v>535678.94304435479</v>
       </c>
       <c r="F3">
         <v>500000</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.1364123550618727</v>
+        <v>0.13641235506187269</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -779,13 +808,13 @@
         <v>1400</v>
       </c>
       <c r="E4">
-        <v>816072.049782366</v>
+        <v>816072.04978236603</v>
       </c>
       <c r="F4">
         <v>800000</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>0.1157556270096463</v>
       </c>
@@ -799,15 +828,15 @@
         <v>1188</v>
       </c>
       <c r="E5">
-        <v>884913.0625394571</v>
+        <v>884913.06253945711</v>
       </c>
       <c r="F5">
         <v>869453</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.4114781253044918</v>
+        <v>0.41147812530449179</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -825,9 +854,9 @@
         <v>1500000</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.1126376303225178</v>
+        <v>0.11263763032251781</v>
       </c>
       <c r="B7" t="s">
         <v>25</v>
@@ -839,15 +868,15 @@
         <v>1156</v>
       </c>
       <c r="E7">
-        <v>897124.7681593318</v>
+        <v>897124.76815933175</v>
       </c>
       <c r="F7">
         <v>898619.6875</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.4262886095683524</v>
+        <v>0.42628860956835241</v>
       </c>
       <c r="B8" t="s">
         <v>25</v>
@@ -859,15 +888,15 @@
         <v>4375</v>
       </c>
       <c r="E8">
-        <v>1063129.868354464</v>
+        <v>1063129.8683544639</v>
       </c>
       <c r="F8">
         <v>930929.4375</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.3561336841079606</v>
+        <v>0.35613368410796059</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -885,9 +914,9 @@
         <v>1043333.375</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.06547793042969892</v>
+        <v>6.5477930429698919E-2</v>
       </c>
       <c r="B10" t="s">
         <v>25</v>
@@ -899,15 +928,15 @@
         <v>672</v>
       </c>
       <c r="E10">
-        <v>3588997.05905878</v>
+        <v>3588997.0590587799</v>
       </c>
       <c r="F10">
         <v>2675000</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>0.01539510864269707</v>
+        <v>1.539510864269707E-2</v>
       </c>
       <c r="B11" t="s">
         <v>25</v>
@@ -919,15 +948,15 @@
         <v>158</v>
       </c>
       <c r="E11">
-        <v>4813543.361550633</v>
+        <v>4813543.3615506329</v>
       </c>
       <c r="F11">
         <v>3245833.375</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>0.02406703692877326</v>
+        <v>2.406703692877326E-2</v>
       </c>
       <c r="B12" t="s">
         <v>25</v>
@@ -939,13 +968,13 @@
         <v>247</v>
       </c>
       <c r="E12">
-        <v>7880210.816295546</v>
+        <v>7880210.8162955455</v>
       </c>
       <c r="F12">
         <v>5358333.5</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>0.2370651856182403</v>
       </c>
@@ -959,15 +988,15 @@
         <v>2433</v>
       </c>
       <c r="E13">
-        <v>921851.8902733893</v>
+        <v>921851.89027338929</v>
       </c>
       <c r="F13">
         <v>700000</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>0.1841566793335282</v>
+        <v>0.18415667933352819</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
@@ -985,9 +1014,9 @@
         <v>833333.3125</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>0.0707395498392283</v>
+        <v>7.0739549839228297E-2</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
@@ -1005,9 +1034,9 @@
         <v>932203</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>0.1284224885511059</v>
+        <v>0.12842248855110591</v>
       </c>
       <c r="B16" t="s">
         <v>32</v>
@@ -1025,9 +1054,9 @@
         <v>1039105.5</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>0.3796160966578973</v>
+        <v>0.37961609665789731</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
@@ -1039,7 +1068,7 @@
         <v>3896</v>
       </c>
       <c r="E17">
-        <v>2290342.222431661</v>
+        <v>2290342.2224316611</v>
       </c>
       <c r="F17">
         <v>1333438.875</v>
@@ -1051,11 +1080,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1084,7 +1113,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1092,7 +1121,7 @@
         <v>4501</v>
       </c>
       <c r="C2">
-        <v>39.09820039991113</v>
+        <v>39.098200399911128</v>
       </c>
       <c r="D2">
         <v>13.01186292429796</v>
@@ -1113,7 +1142,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1124,7 +1153,7 @@
         <v>10.51177777777778</v>
       </c>
       <c r="D3">
-        <v>3.301002285295426</v>
+        <v>3.3010022852954259</v>
       </c>
       <c r="E3">
         <v>11</v>
@@ -1142,7 +1171,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1150,7 +1179,7 @@
         <v>4501</v>
       </c>
       <c r="C4">
-        <v>47.88491446345257</v>
+        <v>47.884914463452567</v>
       </c>
       <c r="D4">
         <v>15.25394219131616</v>
@@ -1171,7 +1200,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1179,10 +1208,10 @@
         <v>4501</v>
       </c>
       <c r="C5">
-        <v>0.4747833814707842</v>
+        <v>0.47478338147078419</v>
       </c>
       <c r="D5">
-        <v>0.4994191990695979</v>
+        <v>0.49941919906959792</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1200,7 +1229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1208,10 +1237,10 @@
         <v>4501</v>
       </c>
       <c r="C6">
-        <v>0.401244167962675</v>
+        <v>0.40124416796267498</v>
       </c>
       <c r="D6">
-        <v>0.4902047265422</v>
+        <v>0.49020472654219999</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1229,7 +1258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1237,10 +1266,10 @@
         <v>4501</v>
       </c>
       <c r="C7">
-        <v>0.3079315707620529</v>
+        <v>0.30793157076205291</v>
       </c>
       <c r="D7">
-        <v>0.4616893719864988</v>
+        <v>0.46168937198649879</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1258,7 +1287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1266,10 +1295,10 @@
         <v>4501</v>
       </c>
       <c r="C8">
-        <v>1674633.798979567</v>
+        <v>1674633.7989795669</v>
       </c>
       <c r="D8">
-        <v>2642172.177935169</v>
+        <v>2642172.1779351691</v>
       </c>
       <c r="E8">
         <v>996453</v>
@@ -1293,11 +1322,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -1317,7 +1346,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0.316</v>
       </c>
@@ -1331,15 +1360,15 @@
         <v>1422</v>
       </c>
       <c r="E2">
-        <v>1050152.868838454</v>
+        <v>1050152.8688384539</v>
       </c>
       <c r="F2">
         <v>936119.6875</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.007777777777777778</v>
+        <v>7.7777777777777784E-3</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
@@ -1351,13 +1380,13 @@
         <v>35</v>
       </c>
       <c r="E3">
-        <v>578646.7053571428</v>
+        <v>578646.70535714284</v>
       </c>
       <c r="F3">
         <v>500000</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>0.1351111111111111</v>
       </c>
@@ -1371,15 +1400,15 @@
         <v>608</v>
       </c>
       <c r="E4">
-        <v>784908.5697214227</v>
+        <v>784908.56972142274</v>
       </c>
       <c r="F4">
         <v>800000</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.1208888888888889</v>
+        <v>0.12088888888888891</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -1391,15 +1420,15 @@
         <v>544</v>
       </c>
       <c r="E5">
-        <v>848200.9420094209</v>
+        <v>848200.94200942095</v>
       </c>
       <c r="F5">
         <v>800000</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.4202222222222222</v>
+        <v>0.42022222222222222</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -1411,15 +1440,15 @@
         <v>1891</v>
       </c>
       <c r="E6">
-        <v>2688787.519004495</v>
+        <v>2688787.5190044949</v>
       </c>
       <c r="F6">
         <v>1552544.375</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.1006443012663853</v>
+        <v>0.10064430126638529</v>
       </c>
       <c r="B7" t="s">
         <v>25</v>
@@ -1431,15 +1460,15 @@
         <v>453</v>
       </c>
       <c r="E7">
-        <v>898948.8351269315</v>
+        <v>898948.83512693155</v>
       </c>
       <c r="F7">
         <v>877033.6875</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.4341257498333704</v>
+        <v>0.43412574983337038</v>
       </c>
       <c r="B8" t="s">
         <v>25</v>
@@ -1451,15 +1480,15 @@
         <v>1954</v>
       </c>
       <c r="E8">
-        <v>1070971.806152844</v>
+        <v>1070971.8061528441</v>
       </c>
       <c r="F8">
         <v>934556.5</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.3590313263719174</v>
+        <v>0.35903132637191743</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -1477,9 +1506,9 @@
         <v>1088211</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.06509664518995778</v>
+        <v>6.509664518995778E-2</v>
       </c>
       <c r="B10" t="s">
         <v>25</v>
@@ -1491,15 +1520,15 @@
         <v>293</v>
       </c>
       <c r="E10">
-        <v>3770477.803754266</v>
+        <v>3770477.8037542659</v>
       </c>
       <c r="F10">
         <v>2500000</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>0.02155076649633415</v>
+        <v>2.155076649633415E-2</v>
       </c>
       <c r="B11" t="s">
         <v>25</v>
@@ -1511,15 +1540,15 @@
         <v>97</v>
       </c>
       <c r="E11">
-        <v>5948266.639175258</v>
+        <v>5948266.6391752576</v>
       </c>
       <c r="F11">
         <v>3450000</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>0.0195512108420351</v>
+        <v>1.9551210842035101E-2</v>
       </c>
       <c r="B12" t="s">
         <v>25</v>
@@ -1531,13 +1560,13 @@
         <v>88</v>
       </c>
       <c r="E12">
-        <v>8632607.436079545</v>
+        <v>8632607.4360795449</v>
       </c>
       <c r="F12">
         <v>6375000</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>0.2463896911797378</v>
       </c>
@@ -1551,15 +1580,15 @@
         <v>1109</v>
       </c>
       <c r="E13">
-        <v>990881.430642048</v>
+        <v>990881.43064204801</v>
       </c>
       <c r="F13">
         <v>700000</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>0.1919573428127083</v>
+        <v>0.19195734281270829</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
@@ -1577,9 +1606,9 @@
         <v>869453</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>0.06820706509664519</v>
+        <v>6.8207065096645189E-2</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
@@ -1591,13 +1620,13 @@
         <v>307</v>
       </c>
       <c r="E15">
-        <v>1291350.673045603</v>
+        <v>1291350.6730456031</v>
       </c>
       <c r="F15">
         <v>957453</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>0.1261941790713175</v>
       </c>
@@ -1617,9 +1646,9 @@
         <v>1005438.84375</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>0.3672517218395912</v>
+        <v>0.36725172183959121</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
@@ -1631,7 +1660,7 @@
         <v>1653</v>
       </c>
       <c r="E17">
-        <v>2413697.35293784</v>
+        <v>2413697.3529378399</v>
       </c>
       <c r="F17">
         <v>1394044.375</v>
@@ -1643,11 +1672,14 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1676,7 +1708,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1684,7 +1716,7 @@
         <v>14764</v>
       </c>
       <c r="C2">
-        <v>38.88817393660255</v>
+        <v>38.888173936602549</v>
       </c>
       <c r="D2">
         <v>13.197837514888</v>
@@ -1705,7 +1737,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1713,10 +1745,10 @@
         <v>14763</v>
       </c>
       <c r="C3">
-        <v>10.50077897446318</v>
+        <v>10.500778974463181</v>
       </c>
       <c r="D3">
-        <v>3.285939973081132</v>
+        <v>3.2859399730811321</v>
       </c>
       <c r="E3">
         <v>11</v>
@@ -1734,7 +1766,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1742,7 +1774,7 @@
         <v>14764</v>
       </c>
       <c r="C4">
-        <v>47.60484963424546</v>
+        <v>47.604849634245461</v>
       </c>
       <c r="D4">
         <v>15.16294725200477</v>
@@ -1763,7 +1795,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1771,10 +1803,10 @@
         <v>14764</v>
       </c>
       <c r="C5">
-        <v>0.4733811975074506</v>
+        <v>0.47338119750745061</v>
       </c>
       <c r="D5">
-        <v>0.4993078465091597</v>
+        <v>0.49930784650915971</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1792,7 +1824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1800,10 +1832,10 @@
         <v>14764</v>
       </c>
       <c r="C6">
-        <v>0.3975887293416419</v>
+        <v>0.39758872934164191</v>
       </c>
       <c r="D6">
-        <v>0.4894161372904047</v>
+        <v>0.48941613729040467</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1821,7 +1853,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1829,10 +1861,10 @@
         <v>14764</v>
       </c>
       <c r="C7">
-        <v>0.2974126253047955</v>
+        <v>0.29741262530479551</v>
       </c>
       <c r="D7">
-        <v>0.4571351111076459</v>
+        <v>0.45713511110764588</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1850,7 +1882,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1858,10 +1890,10 @@
         <v>14764</v>
       </c>
       <c r="C8">
-        <v>1617550.517473352</v>
+        <v>1617550.5174733519</v>
       </c>
       <c r="D8">
-        <v>2431319.117742425</v>
+        <v>2431319.1177424248</v>
       </c>
       <c r="E8">
         <v>992744.6875</v>
@@ -1885,11 +1917,15 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="3" width="8.88671875" customWidth="1"/>
+    <col min="5" max="6" width="8.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -1909,9 +1945,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.3259500101605365</v>
+        <v>0.32595001016053649</v>
       </c>
       <c r="B2" t="s">
         <v>20</v>
@@ -1929,9 +1965,9 @@
         <v>932743</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.006570480254690781</v>
+        <v>6.5704802546907807E-3</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
@@ -1949,7 +1985,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>0.1360157149630834</v>
       </c>
@@ -1963,13 +1999,13 @@
         <v>2008</v>
       </c>
       <c r="E4">
-        <v>806636.0956603275</v>
+        <v>806636.09566032747</v>
       </c>
       <c r="F4">
         <v>800000</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>0.1173203278466436</v>
       </c>
@@ -1983,15 +2019,15 @@
         <v>1732</v>
       </c>
       <c r="E5">
-        <v>873382.2348441109</v>
+        <v>873382.23484411091</v>
       </c>
       <c r="F5">
         <v>843242</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.4141434667750457</v>
+        <v>0.41414346677504571</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -2003,13 +2039,13 @@
         <v>6114</v>
       </c>
       <c r="E6">
-        <v>2568548.285172223</v>
+        <v>2568548.2851722231</v>
       </c>
       <c r="F6">
         <v>1500000</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>0.1089813058791655</v>
       </c>
@@ -2023,15 +2059,15 @@
         <v>1609</v>
       </c>
       <c r="E7">
-        <v>897638.3183994329</v>
+        <v>897638.31839943293</v>
       </c>
       <c r="F7">
         <v>894453</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.4286778650772148</v>
+        <v>0.42867786507721478</v>
       </c>
       <c r="B8" t="s">
         <v>25</v>
@@ -2049,9 +2085,9 @@
         <v>931953</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.3570170685451097</v>
+        <v>0.35701706854510967</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -2069,9 +2105,9 @@
         <v>1055378.625</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.06536169059875373</v>
+        <v>6.5361690598753727E-2</v>
       </c>
       <c r="B10" t="s">
         <v>25</v>
@@ -2083,15 +2119,15 @@
         <v>965</v>
       </c>
       <c r="E10">
-        <v>3644099.502784974</v>
+        <v>3644099.5027849739</v>
       </c>
       <c r="F10">
         <v>2600000</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>0.01727174207531834</v>
+        <v>1.7271742075318341E-2</v>
       </c>
       <c r="B11" t="s">
         <v>25</v>
@@ -2103,15 +2139,15 @@
         <v>255</v>
       </c>
       <c r="E11">
-        <v>5245183.196568628</v>
+        <v>5245183.1965686278</v>
       </c>
       <c r="F11">
         <v>3250000</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>0.02269032782443782</v>
+        <v>2.269032782443782E-2</v>
       </c>
       <c r="B12" t="s">
         <v>25</v>
@@ -2123,15 +2159,15 @@
         <v>335</v>
       </c>
       <c r="E12">
-        <v>8077855.301492537</v>
+        <v>8077855.3014925374</v>
       </c>
       <c r="F12">
         <v>5416666.5</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>0.239907884042265</v>
+        <v>0.23990788404226501</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
@@ -2143,15 +2179,15 @@
         <v>3542</v>
       </c>
       <c r="E13">
-        <v>943465.0354650444</v>
+        <v>943465.03546504444</v>
       </c>
       <c r="F13">
         <v>700000</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>0.1865348144134381</v>
+        <v>0.18653481441343811</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
@@ -2169,9 +2205,9 @@
         <v>842718.4375</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>0.06996748848550528</v>
+        <v>6.9967488485505283E-2</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
@@ -2189,9 +2225,9 @@
         <v>938786.3125</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>0.1277431590354917</v>
+        <v>0.12774315903549169</v>
       </c>
       <c r="B16" t="s">
         <v>32</v>
@@ -2209,9 +2245,9 @@
         <v>1030881.375</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>0.3758466540232999</v>
+        <v>0.37584665402329992</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
@@ -2223,7 +2259,7 @@
         <v>5549</v>
       </c>
       <c r="E17">
-        <v>2327088.668769148</v>
+        <v>2327088.6687691482</v>
       </c>
       <c r="F17">
         <v>1358333.375</v>

</xml_diff>